<commit_message>
liber: 05_IDEAS filled from Buffy Order-3 (21 rows witnessed); Guardian D1 correction; rev1 flag
</commit_message>
<xml_diff>
--- a/liber_status/SOULSMITH_MASTER_STATE.xlsx
+++ b/liber_status/SOULSMITH_MASTER_STATE.xlsx
@@ -22,9 +22,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_TOOLS'!$A$1:$H$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_VENVS'!$A$1:$F$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03_TESTING'!$A$1:$F$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_BUGS'!$A$1:$F$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_IDEAS'!$A$1:$G$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'06_OPEN_ITEMS'!$A$1:$F$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_BUGS'!$A$1:$F$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_IDEAS'!$A$1:$G$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'06_OPEN_ITEMS'!$A$1:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'07_FLEET'!$A$1:$F$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'08_DOCTRINES'!$A$1:$D$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'09_TIMELINE'!$A$1:$D$14</definedName>
@@ -476,7 +476,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>generated_at: 2026-09-26 01:59 UTC  |  source_hash: 17c8505  |  schema: 1.0</t>
+          <t>generated_at: 2026-09-26 02:32 UTC  |  source_hash: 1ca0620  |  schema: 1.0</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -533,7 +533,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>17c8505</t>
+          <t>1ca0620</t>
         </is>
       </c>
     </row>
@@ -555,7 +555,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>17c8505</t>
+          <t>1ca0620</t>
         </is>
       </c>
     </row>
@@ -577,7 +577,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>17c8505</t>
+          <t>1ca0620</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>4 rows</t>
+          <t>7 rows</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -599,7 +599,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>17c8505</t>
+          <t>1ca0620</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2 rows</t>
+          <t>21 rows</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -621,7 +621,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>17c8505</t>
+          <t>1ca0620</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>10 rows</t>
+          <t>11 rows</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -643,7 +643,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>17c8505</t>
+          <t>1ca0620</t>
         </is>
       </c>
     </row>
@@ -665,7 +665,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>17c8505</t>
+          <t>1ca0620</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>17c8505</t>
+          <t>1ca0620</t>
         </is>
       </c>
     </row>
@@ -709,7 +709,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>17c8505</t>
+          <t>1ca0620</t>
         </is>
       </c>
     </row>
@@ -1534,13 +1534,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="49" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="57" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
   </cols>
@@ -1595,7 +1595,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>FIXED same-day per relay PROVISIONAL</t>
+          <t>FIXED same-day syntax }-&gt;) line 118 WITNESSED py_compile clean</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1705,8 +1705,104 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>guardian_dist_empty</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Buffy (48h diagnostic)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>deploy dist/ empty live build in dist_new</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>RESTORED sha256 receipted 21:56</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>shield_test_dead</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Buffy (audit)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>test_soulsmith_shield_v2 imports nonexistent _v3 module</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>OPEN punch #3</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>rcs_import_dash</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Buffy (audit)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>pyMCP_Blender_RCS imports underscore file is dash-named</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>OPEN punch #3</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F5"/>
+  <autoFilter ref="A1:F8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1717,16 +1813,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1769,17 +1865,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PJ-01</t>
+          <t>PJ-1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Buffy</t>
+          <t>Director</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1789,59 +1885,762 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>awaiting Order 3 parcels</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>PROVISIONAL</t>
+          <t>M92 revetment db category flip as pathfinding lever test</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>rig audit pending</t>
+          <t>spawned MAZE_Fortify+DeFort</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BR-01</t>
+          <t>PJ-2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>pickle juice</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>substitute-db template makes any mod statics pathfinding-real</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>breadth test pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PJ-3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>pickle juice</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>MOOSE tasking baseline in maze</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>v3B/C carry telemetry</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PJ-4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>pickle juice</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>gate-keeper flag lattice counts corridor usage</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>v3B wired</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PJ-5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>pickle juice</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>overlap ladder 0cm-2m seam threshold</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>BUILT</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>awaits flight GO2_LADDER_SEAM_v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PJ-6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>pickle juice</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>revetments cut LOS where containers didnt Cover Law</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>v3C LOS lab built</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PJ-7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>pickle juice</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Freebuff restart Lassie metaphor</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>DEAD</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>humor banked</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>PJ-8</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>pickle juice</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>infantry animations terrible</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PARKED</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>engine constraint noted</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>PJ-9</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>pickle juice</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>analyze OBS video with OpenCV-class tools</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>video_lab pipeline proven</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>PJ-10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>pickle juice</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>something fantastic in Tacview</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>RESOLVED</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>became maze verdicts</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PJ-11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Buffy</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>pickle juice</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>lab mods as OvGME packs click-toggle</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>PARKED</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>awaiting Chief</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>PJ-12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Buffy</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>pickle juice</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Qwen3-TTS voice lane agent_voice</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>PARKED</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>qwen_tts module lost see audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>PJ-13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Director+Marco</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>pickle juice</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>TETWR fork-and-gift Fresco way</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>license courtesy first</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>BR-1</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>night tab</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>brainstorm</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>belief-state law probed via v3C fort_wipe/ghost/route</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>design doc owed</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>BR-2</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>night tab</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>brainstorm</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>seam-threading kill-shot: wall hack is seam geometry not LOS fraud</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Cover-Law protocol</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>BR-3</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>night tab</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>brainstorm</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>.fgb mmap grid as runtime belief-grid substrate</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>absorption Phase 0 candidate</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BR-4</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
         <is>
           <t>Buffy</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>brainstorm</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>awaiting Order 3 parcels</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>PROVISIONAL</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>rig audit pending</t>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>unify native build lanes one script or CMake</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>audit punch #1</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BR-5</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Buffy</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>brainstorm</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>flag_scan.py recurring orphan watch beat</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>audit punch #6</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BR-6</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Buffy</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>brainstorm</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>end-of-mission gate-flag dump to log</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>v3B/MONITOR lineage</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>BR-7</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Buffy</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>brainstorm</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Saturation Law as difficulty knob</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>MAZE_LAB_DOCTRINE L5</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>BR-8</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Marco</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>brainstorm</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>absorption doctrine design references clean-room</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>GAVELED</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Phase 0 punch list exists</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G3"/>
+  <autoFilter ref="A1:G22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1852,13 +2651,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="56" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
   </cols>
@@ -1994,7 +2793,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Guardian v3.3 backlog</t>
+          <t>Guardian v3.3 UNBUILT + v3.1 custody repair DONE 09-25</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2009,7 +2808,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>scope</t>
+          <t>v3.3 scope gavel owed</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -2122,7 +2921,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Liber Status sheets 01/02/05</t>
+          <t>Liber Status sheets 01/02</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2132,22 +2931,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Marco</t>
+          <t>Buffy</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Buffy audit data</t>
+          <t>emit CSV per schema v1.0</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+          <t>amber</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
         </is>
       </c>
     </row>
@@ -2215,8 +3014,40 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>rev1 passphrase protection audit</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>security</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>key decrypted batch-mode without passphrase</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F11"/>
+  <autoFilter ref="A1:F12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
rig: parcel_097 — R3 closure, D2 cargo (moose_upflow), Liber 01/02 emitted + schema v1.1, CQD draft + morning report
</commit_message>
<xml_diff>
--- a/liber_status/SOULSMITH_MASTER_STATE.xlsx
+++ b/liber_status/SOULSMITH_MASTER_STATE.xlsx
@@ -19,8 +19,8 @@
     <sheet name="09_TIMELINE" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_TOOLS'!$A$1:$H$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_VENVS'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_TOOLS'!$A$1:$K$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_VENVS'!$A$1:$H$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03_TESTING'!$A$1:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_BUGS'!$A$1:$F$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_IDEAS'!$A$1:$G$22</definedName>
@@ -57,12 +57,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -476,7 +476,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>generated_at: 2026-09-26 02:32 UTC  |  source_hash: 1ca0620  |  schema: 1.0</t>
+          <t>generated_at: 2026-09-26 03:24 UTC  |  source_hash: 1860d58  |  schema: 1.1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -523,7 +523,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0 rows</t>
+          <t>32 rows</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -533,7 +533,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1ca0620</t>
+          <t>1860d58</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0 rows</t>
+          <t>37 rows</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -555,7 +555,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1ca0620</t>
+          <t>1860d58</t>
         </is>
       </c>
     </row>
@@ -577,7 +577,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1ca0620</t>
+          <t>1860d58</t>
         </is>
       </c>
     </row>
@@ -599,7 +599,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1ca0620</t>
+          <t>1860d58</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1ca0620</t>
+          <t>1860d58</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1ca0620</t>
+          <t>1860d58</t>
         </is>
       </c>
     </row>
@@ -665,7 +665,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1ca0620</t>
+          <t>1860d58</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1ca0620</t>
+          <t>1860d58</t>
         </is>
       </c>
     </row>
@@ -709,7 +709,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1ca0620</t>
+          <t>1860d58</t>
         </is>
       </c>
     </row>
@@ -1053,17 +1053,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="54" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="47" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="59" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1107,9 +1110,1524 @@
           <t>last_verified</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>verification_method</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>custody_sha256</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>known_unknown_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>purpose</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>hygiene_flag</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>evidence</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>last_verified</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>verification_method</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>custody_sha256</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>known_unknown_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>vandal_box</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>tools/vandal_box/vandal_box.cpp</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>C++/FSM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>FSM/KB trainer box (C++ twin of vandal_lite)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>exe 09-22 &gt;= src 09-22</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>exe newer than src + audit 1a table</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>fc31e5f63da326bd</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>vandal_lite</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>tools/vandal_lite/</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Python/FSM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>FSM/GOAP/DPARQD engine (11 files, 2107 LOC)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>selftest 17/17 exit 0</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>selftest witness</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>KU-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>acme_moose_cli_v3</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>tools/native_pipe/acme_moose_cli-v3.cpp</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>C++/C2</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Named-pipe C2 CLI (PING/ECHO/STAT/QUIT)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>selftest exit 0</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>pipe selftest witness</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>bc6ac5769bde7e03</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>acme_moose_cli_v2</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>tools/acme_moose_cli-v2.cpp</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>C++/C2</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>v2 CLI -&gt; builds acme_c2_core.exe</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>STALE</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>exe 09-09 &lt; src 09-10</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>audit 1a table</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>ed7607ef9d0c8b7d</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>native_shm_bridge</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>src/native/native_shm_bridge.cpp</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>C++/C2</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Shared-memory bridge</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>exe 09-14 &gt;= src 09-14</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>audit 1a table</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>8f0e41e1d29b0206</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>fortgrid_core</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>src/native/fortgrid_core.cpp</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>C++/LOS</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Fortification-grid fail-closed reader (.fgb)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>smoke 09-25 custody MATCH</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>probe custody MATCH + ray receipt</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>a722789e50aca086</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>modulator_shim</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>src/native/modulator_shim.cpp</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>C++/cognition</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Cognitive modulator shim</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>UNBUILT</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>no artifact ever</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>audit 1a table</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>native_control_injector</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>src/native/native_control_injector.cpp</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>C++/C2</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Stub 6 lines dead since 09-10</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>STUB</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>absorb or delete</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>audit 1c stub triage</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>fortgrid.py</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>tools/fortgrid.py</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Python/maze</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Maze/pathfinding lane core</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>maze lane nightly use</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>audit 1b highlights</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>maze_clip_analyzer.py</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>tools/maze_clip_analyzer.py</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Python/maze</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Wall-clip detection (L5 C3 detector family)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>maze lane nightly use</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>audit 1b highlights</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>KU-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>tacview_forensics_l5.py</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>tools/tacview_forensics_l5.py</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Python/maze</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>KU-3 despair-clip forensics (stall/no-net-progress/clip/skirt)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>v2 refined run 09-26</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>refined two-track run (both series parsed)</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>kill_shot_geometry.py</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>tools/kill_shot_geometry.py</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Python/ballistics</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Seam-threading ballistic geometry (mmap grid)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>py_compile clean post-fix</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>py_compile + witnessed numbers (D8)</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>build_eyes_miz.py</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>tools/build_eyes_miz.py</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Python/miz_builder</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>GO2_EYES_v1.miz builder (v5 generalized SCRIPTS chain)</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>SELF-VERIFY PASS</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>builder self-verify</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>KU-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>build_eyes_batch.py</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>tools/build_eyes_batch.py</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Python/miz_builder</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>E0 B1 batch: 50 miz + manifest + closer</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>B1 built 09-25</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>batch self-verify + manifest</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>KU-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>maze_batch_watchdog.py</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>tools/maze_batch_watchdog.py</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Python/ops</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Batch watchdog v2 (verdicts/restart/shutdown flag-armed)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>flag-armed idle</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>runbook review</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>KU-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>eyes_emit.py</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>tools/eyes_emit.py</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Python/maze_builder</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>MAZE_EYES_v1 emitter (392 occluders embedded)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>pair-verified 39/39</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>eyes_pair_check.py vs lua-5.4.1 selftest</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>map_emit.py</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>tools/map_emit.py</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Python/maze_builder</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MAZE_MAP_v1 poor-man's tacview emitter (75x180 @20 m)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>pair-verified 150/150</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>map_pair_check.py</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>librarian_ingest.py</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>src/librarian_ingest.py</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Python/ingest</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>EPUB/PDF/DOCX ingest -&gt; chromadb</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>BROKEN_PATHWAY</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>8 pkgs uninstalled in every venv</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>audit 1b/flag 4</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>KU-9</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>core_schema.py</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>src/core_schema.py</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Python/schema</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>VirtualSoul pydantic schema</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ALIVE</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>polars</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>audit 1b</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>core_pipeline.py</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>src/core_pipeline.py</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Python/pipeline</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Placeholder one-function stub</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>STUB</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>placeholder by design</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>audit 1c stub triage</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>pyMCP_Blender_RCS_v2</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>tools/pyMCP_Blender_RCS_Server_v2.py</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Python/MCP</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>RCS MCP server</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>BROKEN_IMPORT</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>dash-vs-underscore import bug</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>audit 1b/flag 4</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>soulsmith_mcp_server</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>tools/soulsmith_mcp_server.py</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Python/MCP</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>MCP server (unversioned)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>ALIVE</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>shield test expects _v3 (missing)</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>audit 1b/flag 4</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>test_soulsmith_shield_v2.py</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>src/verification/test_soulsmith_shield_v2.py</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Python/verification</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Shield test harness</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>CANNOT_RUN</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>imports soulsmith_mcp_server_v3 (nonexistent)</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>audit 1b/flag 4</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>qwen_lane_runner.py</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>tools/agent_voice/qwen_lane_runner.py</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Python/voice</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Qwen3-TTS lane runner</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>PARKED</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>module qwen_tts never existed; models present</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>audit 1b/flag 4</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>compile_native_solvers.bat</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>tools/compile_native_solvers.bat</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Build_lane</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Native build bat (knows v2 CLI only)</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>STALE</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>lane fragmentation finding (bat vs .build)</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>audit 1a/flag 1</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>requirements-frozen-2026-09-14.txt</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>requirements-frozen-2026-09-14.txt</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Pin_file</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Frozen requirements (pre-dates opencv/scipy/pydcs adds)</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>STALE</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>core undrifted; pin-gaps due re-freeze</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>audit 1c staleness</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>overnight_diagnostic.py</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>tools/overnight_diagnostic.py</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Python/audit</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Read-only 33-check house diagnostic</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>ALIVE</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>report 5 FAIL/8 WARN/20 OK 09-25</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>diagnostic receipt data/audits/diagnostic_2026-09-25_2220</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>KU-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>gpg_probe.ps1</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>tools/gpg_probe.ps1</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Ops/Custody</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>GPG home + fingerprint probe (GNUPGHOME law)</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>works via GNUPGHOME export</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>ceremony fingerprint match</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>push_lane.sh</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>tools/push_lane.sh</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Ops/lane</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Postal carrier (lane push script)</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>push-verified receipts 09-26</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>lane git receipts</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>flag_scan.py</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>data/audits/build_tool_audit_2026-09-25/flag_scan.py</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Audit/beat</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Orphan/drift/stale-pyc scan (Phase 0 beat candidate)</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>CANDIDATE_BEAT</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Phase 0 punch #6</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>audit adoption recommendation</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>geotiff_emitter.py</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>tools/geotiff_emitter.py</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Python/geo</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>14-band substrate emitter (E7/E7b source)</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>ALIVE</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>substrate witnessed 09-25</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>band inventory receipt</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:K33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1120,15 +2638,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1162,9 +2682,1433 @@
           <t>stale_flag</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>verification_method</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>known_unknown_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>package</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>version</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>venv</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>imported_by</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>orphan_flag</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>stale_flag</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>verification_method</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>known_unknown_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>polars</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1.44.2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>core_schema.py + pipeline tools</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>freeze match 09-14 pin EXACT</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>numpy</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2.5.3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>widespread</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>freeze match 09-14 pin EXACT</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>pydcs</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0.15.0</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>miz builders + pydcs_spawner</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PIN_GAP</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>post-09-14 add unpinned; re-freeze due</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>scipy</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1.18.1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>verification + geo lanes</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PIN_GAP</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>post-09-14 add unpinned; re-freeze due</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>opencv-contrib-python</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>5.0.0.93</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>video_lab/OCR + edm lanes</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PIN_GAP</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>post-09-14 add unpinned; re-freeze due</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>requests</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2.x</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>librarian_ingest.py</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>present per audit flag 4</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>pillow</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2.x</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>librarian_ingest.py + imaging</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>present per audit flag 4</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>chromadb</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>(missing)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>librarian_ingest.py</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>LOST</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>librarian pathway dead until installed</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>KU-9</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>pymupdf</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>(missing)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>librarian_ingest.py</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>LOST</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>librarian pathway dead until installed</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>KU-9</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>pdfplumber</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>(missing)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>librarian_ingest.py</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>LOST</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>librarian pathway dead until installed</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>KU-9</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>pytesseract</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>(missing)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>librarian_ingest.py</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>LOST</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>librarian pathway dead until installed</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>KU-9</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>python-docx</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>(missing)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>librarian_ingest.py</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>LOST</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>librarian pathway dead until installed</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>KU-9</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ebooklib</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>(missing)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>librarian_ingest.py</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>LOST</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>librarian pathway dead until installed</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>KU-9</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>beautifulsoup4</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>(missing)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>librarian_ingest.py</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>LOST</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>librarian pathway dead until installed</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>KU-9</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>mcp</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>(missing)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>pyMCP_* servers + soulsmith_mcp_server</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>LOST</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>never installed in ANY house venv</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>fastmcp</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>(missing)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>soulsmith_mcp_server</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>LOST</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>never installed in ANY house venv</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>torch</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2.14.0+cu126</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>tts_lab</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Qwen3-TTS lane</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>audit 1c census</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>faster-whisper</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>1.2.1</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>tts_lab</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>voice stack</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>aligned across venvs</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ctranslate2</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>4.8.1</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>tts_lab</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>voice stack</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>SKEW</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>forge/acme hold 4.8.2; oldest pin</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>numpy</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>1.26.4</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>acme_librarian</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>librarian pipeline (E: side)</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>SKEW</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>major-version behind forge 2.5.3</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>polars</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>0.20.7</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>acme_librarian</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>librarian pipeline (E: side)</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>SKEW</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>major-version behind forge 1.44.2</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>huggingface_hub</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>1.28.0</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>acme_librarian</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>librarian pipeline (E: side)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>SKEW</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>forge 1.31.0</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>huggingface_hub</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>0.36.2</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>tts_lab</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>voice stack</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>SKEW</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>oldest pin in house</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>onnxruntime</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>1.29.0</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>acme_librarian</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>librarian pipeline (E: side)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>SKEW</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>forge/tts hold 1.30.0</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>sounddevice</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>0.4.6</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>acme_librarian</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>librarian pipeline (E: side)</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>SKEW</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>forge/tts hold 0.5.6</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>tokenizers</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>0.22.2</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>tts_lab</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>voice stack</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>SKEW</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>families divergent</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>deltalake</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>(installed)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>(no house import found)</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>YES_ORPHAN_CANDIDATE</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>purge-candidate list flag 6</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>pyiceberg</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>(installed)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>(no house import found)</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>YES_ORPHAN_CANDIDATE</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>purge-candidate list flag 6</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>connectorx</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>(installed)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>(no house import found)</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>YES_ORPHAN_CANDIDATE</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>purge-candidate list flag 6</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>gevent</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>(installed)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>(no house import found)</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>YES_ORPHAN_CANDIDATE</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>purge-candidate list flag 6</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>altair</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>(installed)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>(no house import found)</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>YES_ORPHAN_CANDIDATE</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>purge-candidate list flag 6</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>xlsxwriter</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>(installed)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>(no house import found)</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>YES_ORPHAN_CANDIDATE</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>one grep each before purge (flag 6)</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>pyinstaller</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>(installed)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Guardian packaging</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>LATENT_BY_DESIGN</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>keep + document (flag 6)</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>pytest</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>(installed)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>test arm</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>LATENT_BY_DESIGN</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>keep + document (flag 6)</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>cupy-cuda12x</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>(installed)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>GPU experiments</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>LATENT_BY_DESIGN</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>keep + document (flag 6)</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>tifffile</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>(installed)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>forge</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>geo/raster stack (terrain_harvest)</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>LATENT_BY_DESIGN</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>keep + document (flag 6)</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1"/>
+  <autoFilter ref="A1:H38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1234,7 +4178,7 @@
           <t>structure-table pathfinder grid test</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1266,7 +4210,7 @@
           <t>A* pathfinding baseline</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1354,7 +4298,7 @@
           <t>designed-thresholds fix applied</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1386,7 +4330,7 @@
           <t>corpus v1.1 execution</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -1418,7 +4362,7 @@
           <t>error net + fail-closed protocol</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1450,7 +4394,7 @@
           <t>run1 anomaly +3514B F: growth</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -1888,7 +4832,7 @@
           <t>M92 revetment db category flip as pathfinding lever test</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -1925,7 +4869,7 @@
           <t>substitute-db template makes any mod statics pathfinding-real</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
@@ -1962,7 +4906,7 @@
           <t>MOOSE tasking baseline in maze</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -1999,7 +4943,7 @@
           <t>gate-keeper flag lattice counts corridor usage</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
@@ -2036,7 +4980,7 @@
           <t>overlap ladder 0cm-2m seam threshold</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>BUILT</t>
         </is>
@@ -2073,7 +5017,7 @@
           <t>revetments cut LOS where containers didnt Cover Law</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
@@ -2110,7 +5054,7 @@
           <t>Freebuff restart Lassie metaphor</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>DEAD</t>
         </is>
@@ -2184,7 +5128,7 @@
           <t>analyze OBS video with OpenCV-class tools</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -2369,7 +5313,7 @@
           <t>belief-state law probed via v3C fort_wipe/ghost/route</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
@@ -2406,7 +5350,7 @@
           <t>seam-threading kill-shot: wall hack is seam geometry not LOS fraud</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
@@ -2443,7 +5387,7 @@
           <t>.fgb mmap grid as runtime belief-grid substrate</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
@@ -2480,7 +5424,7 @@
           <t>unify native build lanes one script or CMake</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
@@ -2517,7 +5461,7 @@
           <t>flag_scan.py recurring orphan watch beat</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
@@ -2554,7 +5498,7 @@
           <t>end-of-mission gate-flag dump to log</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -2591,7 +5535,7 @@
           <t>Saturation Law as difficulty knob</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -2720,7 +5664,7 @@
           <t>red</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -2912,7 +5856,7 @@
           <t>red</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -3040,7 +5984,7 @@
           <t>red</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -3282,7 +6226,7 @@
           <t>rig</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>

</xml_diff>

<commit_message>
cloud: Liber render-check — FIX phantom-header bug (v1.1 CSVs rendered own header as data); true census 148 data rows + 00_INDEX; xlsx re-rendered + copied to Director downloads
</commit_message>
<xml_diff>
--- a/liber_status/SOULSMITH_MASTER_STATE.xlsx
+++ b/liber_status/SOULSMITH_MASTER_STATE.xlsx
@@ -19,8 +19,8 @@
     <sheet name="09_TIMELINE" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_TOOLS'!$A$1:$K$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_VENVS'!$A$1:$H$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_TOOLS'!$A$1:$K$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_VENVS'!$A$1:$H$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03_TESTING'!$A$1:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_BUGS'!$A$1:$F$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_IDEAS'!$A$1:$G$22</definedName>
@@ -476,7 +476,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>generated_at: 2026-09-26 03:24 UTC  |  source_hash: 1860d58  |  schema: 1.1</t>
+          <t>generated_at: 2026-09-26 14:00 UTC  |  source_hash: b854618  |  schema: 1.1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -523,7 +523,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>32 rows</t>
+          <t>31 rows</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -533,7 +533,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1860d58</t>
+          <t>b854618</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>37 rows</t>
+          <t>36 rows</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -555,7 +555,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1860d58</t>
+          <t>b854618</t>
         </is>
       </c>
     </row>
@@ -577,7 +577,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1860d58</t>
+          <t>b854618</t>
         </is>
       </c>
     </row>
@@ -599,7 +599,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1860d58</t>
+          <t>b854618</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1860d58</t>
+          <t>b854618</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1860d58</t>
+          <t>b854618</t>
         </is>
       </c>
     </row>
@@ -665,7 +665,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1860d58</t>
+          <t>b854618</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1860d58</t>
+          <t>b854618</t>
         </is>
       </c>
     </row>
@@ -709,7 +709,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1860d58</t>
+          <t>b854618</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:K32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1129,79 +1129,71 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>vandal_box</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>path</t>
+          <t>tools/vandal_box/vandal_box.cpp</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>C++/FSM</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>purpose</t>
+          <t>FSM/KB trainer box (C++ twin of vandal_lite)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>hygiene_flag</t>
-        </is>
-      </c>
+          <t>CURRENT</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>evidence</t>
+          <t>exe 09-22 &gt;= src 09-22</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>last_verified</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>verification_method</t>
+          <t>exe newer than src + audit 1a table</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>custody_sha256</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>known_unknown_id</t>
-        </is>
-      </c>
+          <t>fc31e5f63da326bd</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>vandal_box</t>
+          <t>vandal_lite</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>tools/vandal_box/vandal_box.cpp</t>
+          <t>tools/vandal_lite/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>C++/FSM</t>
+          <t>Python/FSM</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>FSM/KB trainer box (C++ twin of vandal_lite)</t>
+          <t>FSM/GOAP/DPARQD engine (11 files, 2107 LOC)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1212,7 +1204,7 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>exe 09-22 &gt;= src 09-22</t>
+          <t>selftest 17/17 exit 0</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1222,35 +1214,35 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>exe newer than src + audit 1a table</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>fc31e5f63da326bd</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr"/>
+          <t>selftest witness</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>KU-6</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>vandal_lite</t>
+          <t>acme_moose_cli_v3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>tools/vandal_lite/</t>
+          <t>tools/native_pipe/acme_moose_cli-v3.cpp</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Python/FSM</t>
+          <t>C++/C2</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>FSM/GOAP/DPARQD engine (11 files, 2107 LOC)</t>
+          <t>Named-pipe C2 CLI (PING/ECHO/STAT/QUIT)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1261,7 +1253,7 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>selftest 17/17 exit 0</t>
+          <t>selftest exit 0</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1271,25 +1263,25 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>selftest witness</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>KU-6</t>
-        </is>
-      </c>
+          <t>pipe selftest witness</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>bc6ac5769bde7e03</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>acme_moose_cli_v3</t>
+          <t>acme_moose_cli_v2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>tools/native_pipe/acme_moose_cli-v3.cpp</t>
+          <t>tools/acme_moose_cli-v2.cpp</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1299,18 +1291,18 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Named-pipe C2 CLI (PING/ECHO/STAT/QUIT)</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>CURRENT</t>
+          <t>v2 CLI -&gt; builds acme_c2_core.exe</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>STALE</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>selftest exit 0</t>
+          <t>exe 09-09 &lt; src 09-10</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1320,12 +1312,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>pipe selftest witness</t>
+          <t>audit 1a table</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>bc6ac5769bde7e03</t>
+          <t>ed7607ef9d0c8b7d</t>
         </is>
       </c>
       <c r="K5" t="inlineStr"/>
@@ -1333,12 +1325,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>acme_moose_cli_v2</t>
+          <t>native_shm_bridge</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>tools/acme_moose_cli-v2.cpp</t>
+          <t>src/native/native_shm_bridge.cpp</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1348,18 +1340,18 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>v2 CLI -&gt; builds acme_c2_core.exe</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>STALE</t>
+          <t>Shared-memory bridge</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>CURRENT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>exe 09-09 &lt; src 09-10</t>
+          <t>exe 09-14 &gt;= src 09-14</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1374,7 +1366,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>ed7607ef9d0c8b7d</t>
+          <t>8f0e41e1d29b0206</t>
         </is>
       </c>
       <c r="K6" t="inlineStr"/>
@@ -1382,22 +1374,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>native_shm_bridge</t>
+          <t>fortgrid_core</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>src/native/native_shm_bridge.cpp</t>
+          <t>src/native/fortgrid_core.cpp</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>C++/C2</t>
+          <t>C++/LOS</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Shared-memory bridge</t>
+          <t>Fortification-grid fail-closed reader (.fgb)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1408,7 +1400,7 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>exe 09-14 &gt;= src 09-14</t>
+          <t>smoke 09-25 custody MATCH</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1418,12 +1410,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>audit 1a table</t>
+          <t>probe custody MATCH + ray receipt</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>8f0e41e1d29b0206</t>
+          <t>a722789e50aca086</t>
         </is>
       </c>
       <c r="K7" t="inlineStr"/>
@@ -1431,33 +1423,33 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>fortgrid_core</t>
+          <t>modulator_shim</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>src/native/fortgrid_core.cpp</t>
+          <t>src/native/modulator_shim.cpp</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>C++/LOS</t>
+          <t>C++/cognition</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Fortification-grid fail-closed reader (.fgb)</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>CURRENT</t>
+          <t>Cognitive modulator shim</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>UNBUILT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>smoke 09-25 custody MATCH</t>
+          <t>no artifact ever</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1467,46 +1459,42 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>probe custody MATCH + ray receipt</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>a722789e50aca086</t>
-        </is>
-      </c>
+          <t>audit 1a table</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>modulator_shim</t>
+          <t>native_control_injector</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>src/native/modulator_shim.cpp</t>
+          <t>src/native/native_control_injector.cpp</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>C++/cognition</t>
+          <t>C++/C2</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Cognitive modulator shim</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>UNBUILT</t>
+          <t>Stub 6 lines dead since 09-10</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>STUB</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>no artifact ever</t>
+          <t>absorb or delete</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1516,7 +1504,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>audit 1a table</t>
+          <t>audit 1c stub triage</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -1525,33 +1513,33 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>native_control_injector</t>
+          <t>fortgrid.py</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>src/native/native_control_injector.cpp</t>
+          <t>tools/fortgrid.py</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>C++/C2</t>
+          <t>Python/maze</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Stub 6 lines dead since 09-10</t>
+          <t>Maze/pathfinding lane core</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>STUB</t>
+          <t>CURRENT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>absorb or delete</t>
+          <t>maze lane nightly use</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1561,7 +1549,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>audit 1c stub triage</t>
+          <t>audit 1b highlights</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -1570,12 +1558,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>fortgrid.py</t>
+          <t>maze_clip_analyzer.py</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>tools/fortgrid.py</t>
+          <t>tools/maze_clip_analyzer.py</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1585,7 +1573,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Maze/pathfinding lane core</t>
+          <t>Wall-clip detection (L5 C3 detector family)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1610,17 +1598,21 @@
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>KU-3</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>maze_clip_analyzer.py</t>
+          <t>tacview_forensics_l5.py</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>tools/maze_clip_analyzer.py</t>
+          <t>tools/tacview_forensics_l5.py</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1630,7 +1622,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Wall-clip detection (L5 C3 detector family)</t>
+          <t>KU-3 despair-clip forensics (stall/no-net-progress/clip/skirt)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1641,45 +1633,41 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>maze lane nightly use</t>
+          <t>v2 refined run 09-26</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>audit 1b highlights</t>
+          <t>refined two-track run (both series parsed)</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>KU-3</t>
-        </is>
-      </c>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>tacview_forensics_l5.py</t>
+          <t>kill_shot_geometry.py</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>tools/tacview_forensics_l5.py</t>
+          <t>tools/kill_shot_geometry.py</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Python/maze</t>
+          <t>Python/ballistics</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>KU-3 despair-clip forensics (stall/no-net-progress/clip/skirt)</t>
+          <t>Seam-threading ballistic geometry (mmap grid)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1690,17 +1678,17 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>v2 refined run 09-26</t>
+          <t>py_compile clean post-fix</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>refined two-track run (both series parsed)</t>
+          <t>py_compile + witnessed numbers (D8)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
@@ -1709,22 +1697,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>kill_shot_geometry.py</t>
+          <t>build_eyes_miz.py</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>tools/kill_shot_geometry.py</t>
+          <t>tools/build_eyes_miz.py</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Python/ballistics</t>
+          <t>Python/miz_builder</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Seam-threading ballistic geometry (mmap grid)</t>
+          <t>GO2_EYES_v1.miz builder (v5 generalized SCRIPTS chain)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1735,7 +1723,7 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>py_compile clean post-fix</t>
+          <t>SELF-VERIFY PASS</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1745,21 +1733,25 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>py_compile + witnessed numbers (D8)</t>
+          <t>builder self-verify</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>KU-10</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>build_eyes_miz.py</t>
+          <t>build_eyes_batch.py</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>tools/build_eyes_miz.py</t>
+          <t>tools/build_eyes_batch.py</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1769,7 +1761,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>GO2_EYES_v1.miz builder (v5 generalized SCRIPTS chain)</t>
+          <t>E0 B1 batch: 50 miz + manifest + closer</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1780,7 +1772,7 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>SELF-VERIFY PASS</t>
+          <t>B1 built 09-25</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1790,7 +1782,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>builder self-verify</t>
+          <t>batch self-verify + manifest</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
@@ -1803,22 +1795,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>build_eyes_batch.py</t>
+          <t>maze_batch_watchdog.py</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>tools/build_eyes_batch.py</t>
+          <t>tools/maze_batch_watchdog.py</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Python/miz_builder</t>
+          <t>Python/ops</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>E0 B1 batch: 50 miz + manifest + closer</t>
+          <t>Batch watchdog v2 (verdicts/restart/shutdown flag-armed)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1829,7 +1821,7 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>B1 built 09-25</t>
+          <t>flag-armed idle</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1839,7 +1831,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>batch self-verify + manifest</t>
+          <t>runbook review</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
@@ -1852,22 +1844,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>maze_batch_watchdog.py</t>
+          <t>eyes_emit.py</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>tools/maze_batch_watchdog.py</t>
+          <t>tools/eyes_emit.py</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Python/ops</t>
+          <t>Python/maze_builder</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Batch watchdog v2 (verdicts/restart/shutdown flag-armed)</t>
+          <t>MAZE_EYES_v1 emitter (392 occluders embedded)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1878,7 +1870,7 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>flag-armed idle</t>
+          <t>pair-verified 39/39</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1888,25 +1880,21 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>runbook review</t>
+          <t>eyes_pair_check.py vs lua-5.4.1 selftest</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>KU-10</t>
-        </is>
-      </c>
+      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>eyes_emit.py</t>
+          <t>map_emit.py</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>tools/eyes_emit.py</t>
+          <t>tools/map_emit.py</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1916,7 +1904,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>MAZE_EYES_v1 emitter (392 occluders embedded)</t>
+          <t>MAZE_MAP_v1 poor-man's tacview emitter (75x180 @20 m)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1927,7 +1915,7 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>pair-verified 39/39</t>
+          <t>pair-verified 150/150</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1937,7 +1925,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>eyes_pair_check.py vs lua-5.4.1 selftest</t>
+          <t>map_pair_check.py</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -1946,33 +1934,33 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>map_emit.py</t>
+          <t>librarian_ingest.py</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>tools/map_emit.py</t>
+          <t>src/librarian_ingest.py</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Python/maze_builder</t>
+          <t>Python/ingest</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>MAZE_MAP_v1 poor-man's tacview emitter (75x180 @20 m)</t>
+          <t>EPUB/PDF/DOCX ingest -&gt; chromadb</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>CURRENT</t>
+          <t>BROKEN_PATHWAY</t>
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>pair-verified 150/150</t>
+          <t>8 pkgs uninstalled in every venv</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1982,42 +1970,46 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>map_pair_check.py</t>
+          <t>audit 1b/flag 4</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>KU-9</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>librarian_ingest.py</t>
+          <t>core_schema.py</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>src/librarian_ingest.py</t>
+          <t>src/core_schema.py</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Python/ingest</t>
+          <t>Python/schema</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>EPUB/PDF/DOCX ingest -&gt; chromadb</t>
+          <t>VirtualSoul pydantic schema</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BROKEN_PATHWAY</t>
+          <t>ALIVE</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>8 pkgs uninstalled in every venv</t>
+          <t>polars</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2027,46 +2019,42 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>audit 1b/flag 4</t>
+          <t>audit 1b</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>KU-9</t>
-        </is>
-      </c>
+      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>core_schema.py</t>
+          <t>core_pipeline.py</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>src/core_schema.py</t>
+          <t>src/core_pipeline.py</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Python/schema</t>
+          <t>Python/pipeline</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>VirtualSoul pydantic schema</t>
+          <t>Placeholder one-function stub</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ALIVE</t>
+          <t>STUB</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>polars</t>
+          <t>placeholder by design</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2076,7 +2064,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>audit 1b</t>
+          <t>audit 1c stub triage</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -2085,33 +2073,33 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>core_pipeline.py</t>
+          <t>pyMCP_Blender_RCS_v2</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>src/core_pipeline.py</t>
+          <t>tools/pyMCP_Blender_RCS_Server_v2.py</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Python/pipeline</t>
+          <t>Python/MCP</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Placeholder one-function stub</t>
+          <t>RCS MCP server</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>STUB</t>
+          <t>BROKEN_IMPORT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>placeholder by design</t>
+          <t>dash-vs-underscore import bug</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2121,7 +2109,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>audit 1c stub triage</t>
+          <t>audit 1b/flag 4</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
@@ -2130,12 +2118,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>pyMCP_Blender_RCS_v2</t>
+          <t>soulsmith_mcp_server</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>tools/pyMCP_Blender_RCS_Server_v2.py</t>
+          <t>tools/soulsmith_mcp_server.py</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2145,18 +2133,18 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>RCS MCP server</t>
+          <t>MCP server (unversioned)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>BROKEN_IMPORT</t>
+          <t>ALIVE</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>dash-vs-underscore import bug</t>
+          <t>shield test expects _v3 (missing)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2175,33 +2163,33 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>soulsmith_mcp_server</t>
+          <t>test_soulsmith_shield_v2.py</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>tools/soulsmith_mcp_server.py</t>
+          <t>src/verification/test_soulsmith_shield_v2.py</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Python/MCP</t>
+          <t>Python/verification</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>MCP server (unversioned)</t>
+          <t>Shield test harness</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>ALIVE</t>
+          <t>CANNOT_RUN</t>
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>shield test expects _v3 (missing)</t>
+          <t>imports soulsmith_mcp_server_v3 (nonexistent)</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2220,33 +2208,33 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>test_soulsmith_shield_v2.py</t>
+          <t>qwen_lane_runner.py</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>src/verification/test_soulsmith_shield_v2.py</t>
+          <t>tools/agent_voice/qwen_lane_runner.py</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Python/verification</t>
+          <t>Python/voice</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Shield test harness</t>
+          <t>Qwen3-TTS lane runner</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>CANNOT_RUN</t>
+          <t>PARKED</t>
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>imports soulsmith_mcp_server_v3 (nonexistent)</t>
+          <t>module qwen_tts never existed; models present</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2265,33 +2253,33 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>qwen_lane_runner.py</t>
+          <t>compile_native_solvers.bat</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>tools/agent_voice/qwen_lane_runner.py</t>
+          <t>tools/compile_native_solvers.bat</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Python/voice</t>
+          <t>Build_lane</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Qwen3-TTS lane runner</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>PARKED</t>
+          <t>Native build bat (knows v2 CLI only)</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>STALE</t>
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>module qwen_tts never existed; models present</t>
+          <t>lane fragmentation finding (bat vs .build)</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2301,7 +2289,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>audit 1b/flag 4</t>
+          <t>audit 1a/flag 1</t>
         </is>
       </c>
       <c r="J26" t="inlineStr"/>
@@ -2310,22 +2298,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>compile_native_solvers.bat</t>
+          <t>requirements-frozen-2026-09-14.txt</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>tools/compile_native_solvers.bat</t>
+          <t>requirements-frozen-2026-09-14.txt</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Build_lane</t>
+          <t>Pin_file</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Native build bat (knows v2 CLI only)</t>
+          <t>Frozen requirements (pre-dates opencv/scipy/pydcs adds)</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -2336,7 +2324,7 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>lane fragmentation finding (bat vs .build)</t>
+          <t>core undrifted; pin-gaps due re-freeze</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2346,7 +2334,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>audit 1a/flag 1</t>
+          <t>audit 1c staleness</t>
         </is>
       </c>
       <c r="J27" t="inlineStr"/>
@@ -2355,33 +2343,33 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>requirements-frozen-2026-09-14.txt</t>
+          <t>overnight_diagnostic.py</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>requirements-frozen-2026-09-14.txt</t>
+          <t>tools/overnight_diagnostic.py</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Pin_file</t>
+          <t>Python/audit</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Frozen requirements (pre-dates opencv/scipy/pydcs adds)</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>STALE</t>
+          <t>Read-only 33-check house diagnostic</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>ALIVE</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>core undrifted; pin-gaps due re-freeze</t>
+          <t>report 5 FAIL/8 WARN/20 OK 09-25</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2391,42 +2379,46 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>audit 1c staleness</t>
+          <t>diagnostic receipt data/audits/diagnostic_2026-09-25_2220</t>
         </is>
       </c>
       <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>KU-11</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>overnight_diagnostic.py</t>
+          <t>gpg_probe.ps1</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>tools/overnight_diagnostic.py</t>
+          <t>tools/gpg_probe.ps1</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Python/audit</t>
+          <t>Ops/Custody</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Read-only 33-check house diagnostic</t>
+          <t>GPG home + fingerprint probe (GNUPGHOME law)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ALIVE</t>
+          <t>CURRENT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>report 5 FAIL/8 WARN/20 OK 09-25</t>
+          <t>works via GNUPGHOME export</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2436,35 +2428,31 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>diagnostic receipt data/audits/diagnostic_2026-09-25_2220</t>
+          <t>ceremony fingerprint match</t>
         </is>
       </c>
       <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>KU-11</t>
-        </is>
-      </c>
+      <c r="K29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>gpg_probe.ps1</t>
+          <t>push_lane.sh</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>tools/gpg_probe.ps1</t>
+          <t>tools/push_lane.sh</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Ops/Custody</t>
+          <t>Ops/lane</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>GPG home + fingerprint probe (GNUPGHOME law)</t>
+          <t>Postal carrier (lane push script)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2475,17 +2463,17 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>works via GNUPGHOME export</t>
+          <t>push-verified receipts 09-26</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>ceremony fingerprint match</t>
+          <t>lane git receipts</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
@@ -2494,43 +2482,43 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>push_lane.sh</t>
+          <t>flag_scan.py</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>tools/push_lane.sh</t>
+          <t>data/audits/build_tool_audit_2026-09-25/flag_scan.py</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Ops/lane</t>
+          <t>Audit/beat</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Postal carrier (lane push script)</t>
+          <t>Orphan/drift/stale-pyc scan (Phase 0 beat candidate)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>CURRENT</t>
+          <t>CANDIDATE_BEAT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>push-verified receipts 09-26</t>
+          <t>Phase 0 punch #6</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>lane git receipts</t>
+          <t>audit adoption recommendation</t>
         </is>
       </c>
       <c r="J31" t="inlineStr"/>
@@ -2539,33 +2527,33 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>flag_scan.py</t>
+          <t>geotiff_emitter.py</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>data/audits/build_tool_audit_2026-09-25/flag_scan.py</t>
+          <t>tools/geotiff_emitter.py</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Audit/beat</t>
+          <t>Python/geo</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Orphan/drift/stale-pyc scan (Phase 0 beat candidate)</t>
+          <t>14-band substrate emitter (E7/E7b source)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>CANDIDATE_BEAT</t>
+          <t>ALIVE</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Phase 0 punch #6</t>
+          <t>substrate witnessed 09-25</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2575,59 +2563,14 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>audit adoption recommendation</t>
+          <t>band inventory receipt</t>
         </is>
       </c>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>geotiff_emitter.py</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>tools/geotiff_emitter.py</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Python/geo</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>14-band substrate emitter (E7/E7b source)</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>ALIVE</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>substrate witnessed 09-25</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>band inventory receipt</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K33"/>
+  <autoFilter ref="A1:K32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2638,7 +2581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -2696,54 +2639,50 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>package</t>
+          <t>polars</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>1.44.2</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>venv</t>
+          <t>forge</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>imported_by</t>
+          <t>core_schema.py + pipeline tools</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>orphan_flag</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>stale_flag</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>verification_method</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>known_unknown_id</t>
-        </is>
-      </c>
+          <t>freeze match 09-14 pin EXACT</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>polars</t>
+          <t>numpy</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1.44.2</t>
+          <t>2.5.3</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2753,7 +2692,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>core_schema.py + pipeline tools</t>
+          <t>widespread</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -2776,12 +2715,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>numpy</t>
+          <t>pydcs</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2.5.3</t>
+          <t>0.15.0</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2791,7 +2730,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>widespread</t>
+          <t>miz builders + pydcs_spawner</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -2801,12 +2740,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>PIN_GAP</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>freeze match 09-14 pin EXACT</t>
+          <t>post-09-14 add unpinned; re-freeze due</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -2814,12 +2753,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>pydcs</t>
+          <t>scipy</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0.15.0</t>
+          <t>1.18.1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2829,7 +2768,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>miz builders + pydcs_spawner</t>
+          <t>verification + geo lanes</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -2852,12 +2791,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>scipy</t>
+          <t>opencv-contrib-python</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1.18.1</t>
+          <t>5.0.0.93</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2867,7 +2806,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>verification + geo lanes</t>
+          <t>video_lab/OCR + edm lanes</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -2890,12 +2829,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>opencv-contrib-python</t>
+          <t>requests</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>5.0.0.93</t>
+          <t>2.x</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2905,7 +2844,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>video_lab/OCR + edm lanes</t>
+          <t>librarian_ingest.py</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -2915,12 +2854,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>PIN_GAP</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>post-09-14 add unpinned; re-freeze due</t>
+          <t>present per audit flag 4</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
@@ -2928,7 +2867,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>requests</t>
+          <t>pillow</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2943,7 +2882,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>librarian_ingest.py</t>
+          <t>librarian_ingest.py + imaging</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -2966,12 +2905,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>pillow</t>
+          <t>chromadb</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2.x</t>
+          <t>(missing)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2981,30 +2920,34 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>librarian_ingest.py + imaging</t>
+          <t>librarian_ingest.py</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>LOST</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>present per audit flag 4</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
+          <t>librarian pathway dead until installed</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>KU-9</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>chromadb</t>
+          <t>pymupdf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -3046,7 +2989,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>pymupdf</t>
+          <t>pdfplumber</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -3088,7 +3031,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>pdfplumber</t>
+          <t>pytesseract</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -3130,7 +3073,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>pytesseract</t>
+          <t>python-docx</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -3172,7 +3115,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>python-docx</t>
+          <t>ebooklib</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -3214,7 +3157,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ebooklib</t>
+          <t>beautifulsoup4</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3256,7 +3199,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>beautifulsoup4</t>
+          <t>mcp</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3271,7 +3214,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>librarian_ingest.py</t>
+          <t>pyMCP_* servers + soulsmith_mcp_server</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -3286,19 +3229,15 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>librarian pathway dead until installed</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>KU-9</t>
-        </is>
-      </c>
+          <t>never installed in ANY house venv</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>mcp</t>
+          <t>fastmcp</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3313,7 +3252,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>pyMCP_* servers + soulsmith_mcp_server</t>
+          <t>soulsmith_mcp_server</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -3336,37 +3275,37 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>fastmcp</t>
+          <t>torch</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>(missing)</t>
+          <t>2.14.0+cu126</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>forge</t>
+          <t>tts_lab</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>soulsmith_mcp_server</t>
+          <t>Qwen3-TTS lane</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>LOST</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>never installed in ANY house venv</t>
+          <t>audit 1c census</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
@@ -3374,12 +3313,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>torch</t>
+          <t>faster-whisper</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2.14.0+cu126</t>
+          <t>1.2.1</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -3389,7 +3328,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Qwen3-TTS lane</t>
+          <t>voice stack</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -3404,7 +3343,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>audit 1c census</t>
+          <t>aligned across venvs</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -3412,12 +3351,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>faster-whisper</t>
+          <t>ctranslate2</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1.2.1</t>
+          <t>4.8.1</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3437,12 +3376,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>SKEW</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>aligned across venvs</t>
+          <t>forge/acme hold 4.8.2; oldest pin</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
@@ -3450,22 +3389,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ctranslate2</t>
+          <t>numpy</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>4.8.1</t>
+          <t>1.26.4</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>tts_lab</t>
+          <t>acme_librarian</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>voice stack</t>
+          <t>librarian pipeline (E: side)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -3480,7 +3419,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>forge/acme hold 4.8.2; oldest pin</t>
+          <t>major-version behind forge 2.5.3</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -3488,12 +3427,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>numpy</t>
+          <t>polars</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1.26.4</t>
+          <t>0.20.7</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -3518,7 +3457,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>major-version behind forge 2.5.3</t>
+          <t>major-version behind forge 1.44.2</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -3526,12 +3465,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>polars</t>
+          <t>huggingface_hub</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0.20.7</t>
+          <t>1.28.0</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -3556,7 +3495,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>major-version behind forge 1.44.2</t>
+          <t>forge 1.31.0</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
@@ -3569,17 +3508,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>1.28.0</t>
+          <t>0.36.2</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>acme_librarian</t>
+          <t>tts_lab</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>librarian pipeline (E: side)</t>
+          <t>voice stack</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -3594,7 +3533,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>forge 1.31.0</t>
+          <t>oldest pin in house</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -3602,22 +3541,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>huggingface_hub</t>
+          <t>onnxruntime</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0.36.2</t>
+          <t>1.29.0</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>tts_lab</t>
+          <t>acme_librarian</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>voice stack</t>
+          <t>librarian pipeline (E: side)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -3632,7 +3571,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>oldest pin in house</t>
+          <t>forge/tts hold 1.30.0</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
@@ -3640,12 +3579,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>onnxruntime</t>
+          <t>sounddevice</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>1.29.0</t>
+          <t>0.4.6</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3670,7 +3609,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>forge/tts hold 1.30.0</t>
+          <t>forge/tts hold 0.5.6</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
@@ -3678,22 +3617,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>sounddevice</t>
+          <t>tokenizers</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0.4.6</t>
+          <t>0.22.2</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>acme_librarian</t>
+          <t>tts_lab</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>librarian pipeline (E: side)</t>
+          <t>voice stack</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -3708,7 +3647,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>forge/tts hold 0.5.6</t>
+          <t>families divergent</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
@@ -3716,37 +3655,33 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>tokenizers</t>
+          <t>deltalake</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0.22.2</t>
+          <t>(installed)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>tts_lab</t>
+          <t>forge</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>voice stack</t>
+          <t>(no house import found)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>SKEW</t>
-        </is>
-      </c>
+          <t>YES_ORPHAN_CANDIDATE</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>families divergent</t>
+          <t>purge-candidate list flag 6</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
@@ -3754,7 +3689,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>deltalake</t>
+          <t>pyiceberg</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3788,7 +3723,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>pyiceberg</t>
+          <t>connectorx</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3822,7 +3757,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>connectorx</t>
+          <t>gevent</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3856,7 +3791,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>gevent</t>
+          <t>altair</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3890,7 +3825,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>altair</t>
+          <t>xlsxwriter</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3916,7 +3851,7 @@
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>purge-candidate list flag 6</t>
+          <t>one grep each before purge (flag 6)</t>
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
@@ -3924,7 +3859,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>xlsxwriter</t>
+          <t>pyinstaller</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3939,18 +3874,22 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>(no house import found)</t>
+          <t>Guardian packaging</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>YES_ORPHAN_CANDIDATE</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr"/>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>LATENT_BY_DESIGN</t>
+        </is>
+      </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>one grep each before purge (flag 6)</t>
+          <t>keep + document (flag 6)</t>
         </is>
       </c>
       <c r="H34" t="inlineStr"/>
@@ -3958,7 +3897,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>pyinstaller</t>
+          <t>pytest</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3973,7 +3912,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Guardian packaging</t>
+          <t>test arm</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3996,7 +3935,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>pytest</t>
+          <t>cupy-cuda12x</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4011,7 +3950,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>test arm</t>
+          <t>GPU experiments</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -4034,7 +3973,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>cupy-cuda12x</t>
+          <t>tifffile</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4049,7 +3988,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>GPU experiments</t>
+          <t>geo/raster stack (terrain_harvest)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -4069,46 +4008,8 @@
       </c>
       <c r="H37" t="inlineStr"/>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>tifffile</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>(installed)</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>forge</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>geo/raster stack (terrain_harvest)</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>LATENT_BY_DESIGN</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>keep + document (flag 6)</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H38"/>
+  <autoFilter ref="A1:H37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
cloud: 06_OPEN_ITEMS morning reconcile — 6 closures witnessed (rig-alive, Phase 0, 01/02, generator, vault backup) + 3 new (trainer gavels, MOOSE scrubs, Watch Card merge)
</commit_message>
<xml_diff>
--- a/liber_status/SOULSMITH_MASTER_STATE.xlsx
+++ b/liber_status/SOULSMITH_MASTER_STATE.xlsx
@@ -24,7 +24,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03_TESTING'!$A$1:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_BUGS'!$A$1:$F$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_IDEAS'!$A$1:$G$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'06_OPEN_ITEMS'!$A$1:$F$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'06_OPEN_ITEMS'!$A$1:$F$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'07_FLEET'!$A$1:$F$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'08_DOCTRINES'!$A$1:$D$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'09_TIMELINE'!$A$1:$D$14</definedName>
@@ -476,7 +476,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>generated_at: 2026-09-26 14:00 UTC  |  source_hash: b854618  |  schema: 1.1</t>
+          <t>generated_at: 2026-09-26 14:02 UTC  |  source_hash: 255f98d  |  schema: 1.1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -533,7 +533,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>b854618</t>
+          <t>255f98d</t>
         </is>
       </c>
     </row>
@@ -555,7 +555,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>b854618</t>
+          <t>255f98d</t>
         </is>
       </c>
     </row>
@@ -577,7 +577,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>b854618</t>
+          <t>255f98d</t>
         </is>
       </c>
     </row>
@@ -599,7 +599,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>b854618</t>
+          <t>255f98d</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>b854618</t>
+          <t>255f98d</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>11 rows</t>
+          <t>15 rows</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -643,7 +643,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>b854618</t>
+          <t>255f98d</t>
         </is>
       </c>
     </row>
@@ -665,7 +665,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>b854618</t>
+          <t>255f98d</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>b854618</t>
+          <t>255f98d</t>
         </is>
       </c>
     </row>
@@ -709,7 +709,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>b854618</t>
+          <t>255f98d</t>
         </is>
       </c>
     </row>
@@ -5496,15 +5496,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5562,12 +5562,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>CLOSED 09-26 — D5: rig went quiet not shipwreck; lane push gap, parcels 089-099 crossed</t>
         </is>
       </c>
     </row>
@@ -5754,12 +5754,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>CLOSED-REGISTERED 09-26 — dev doc 43b2631, 8 items witnessed+sequenced</t>
         </is>
       </c>
     </row>
@@ -5786,12 +5786,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>amber</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>CLOSED 09-26 — emitted v1.1 (31+36 rows), render-check PASS after phantom-header fix 4f7f3d7</t>
         </is>
       </c>
     </row>
@@ -5821,9 +5821,9 @@
           <t>green</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>IN_PROGRESS</t>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>CLOSED 09-26 — built + v1.1 header fix shipped</t>
         </is>
       </c>
     </row>
@@ -5887,12 +5887,140 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN — RED stands; key recovered 09-26 but batch-mode decrypt still unaudited</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>trainer Q1/Q4/Q5 gavels</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>planning</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Marco recs DELIVERED cloud-104</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>amber</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>PENDING — Q2/Q3/Q6 close-ready on countersigns</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>MOOSE upflow submission</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>upstream</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>conformity CONDITIONAL PASS cloud-103; 2 scrubs owed rig-side</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>amber</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>PENDING — scrub C1 rig paths, C2 doctrine voice</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Watch Card v1 merge + adoption</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>doctrine</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Buffy+Director</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Marco v1 delta cloud-101 delivered</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>amber</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>PENDING — merge then Director gavel</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>vault single-copy risk</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>infrastructure</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Marco</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>CLOSED 09-26 — encrypted backup to lane cloud-102 (7abe6dff)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F12"/>
+  <autoFilter ref="A1:F16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>